<commit_message>
chore: update project structure and documentation
- Add LICENSE file with MIT License.
- Introduce mkdocs.yml for documentation management.
- Create GitHub Actions workflow for automatic documentation deployment.
- Add new documentation files for bus data assignment, configuration definition, copyright, examples, and grid data access.
- Remove outdated config_definition.md and tx123bt_workflow.md files.
- Update .gitignore to include new directories and files.
</commit_message>
<xml_diff>
--- a/examples/14bus_uc/14bus_config.xlsx
+++ b/examples/14bus_uc/14bus_config.xlsx
@@ -10,10 +10,10 @@
     <sheet name="bus" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="gen" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="branch" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="gencost" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="solar" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="wind" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="load" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="solar" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="wind" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="load" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="__metadata__" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1086,7 +1086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:AB3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1142,42 +1142,92 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>COST_MODEL</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>COST_STARTUP</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>COST_SHUTDOWN</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>COST_ORDER</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>COST_SECOND</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>COST_FIRST</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>COST_ZERO</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>RAMP_UP</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>RAMP_DOWN</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>RAMP_STARTUP</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>RAMP_SHUTDOWN</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>RAMP_UP_RD</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>RAMP_DOWN_RD</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>MIN_ON_TIME</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>MIN_OFF_TIME</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>COST_STORAGE</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>COST_RD_UP</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>COST_RD_DOWN</t>
         </is>
       </c>
     </row>
@@ -1213,28 +1263,58 @@
         <v>16</v>
       </c>
       <c r="K2" t="n">
+        <v>2</v>
+      </c>
+      <c r="L2" t="n">
+        <v>60</v>
+      </c>
+      <c r="M2" t="n">
+        <v>10</v>
+      </c>
+      <c r="N2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>20</v>
+      </c>
+      <c r="R2" t="n">
         <v>40</v>
       </c>
-      <c r="L2" t="n">
+      <c r="S2" t="n">
         <v>80</v>
       </c>
-      <c r="M2" t="n">
+      <c r="T2" t="n">
         <v>80</v>
       </c>
-      <c r="N2" t="n">
+      <c r="U2" t="n">
         <v>80</v>
       </c>
-      <c r="O2" t="n">
+      <c r="V2" t="n">
         <v>16</v>
       </c>
-      <c r="P2" t="n">
+      <c r="W2" t="n">
         <v>40</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="X2" t="n">
         <v>5</v>
       </c>
-      <c r="R2" t="n">
+      <c r="Y2" t="n">
         <v>2</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>20</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -1269,28 +1349,58 @@
         <v>10</v>
       </c>
       <c r="K3" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="L3" t="n">
         <v>50</v>
       </c>
       <c r="M3" t="n">
+        <v>5</v>
+      </c>
+      <c r="N3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>40</v>
+      </c>
+      <c r="R3" t="n">
+        <v>25</v>
+      </c>
+      <c r="S3" t="n">
         <v>50</v>
       </c>
-      <c r="N3" t="n">
+      <c r="T3" t="n">
         <v>50</v>
       </c>
-      <c r="O3" t="n">
+      <c r="U3" t="n">
+        <v>50</v>
+      </c>
+      <c r="V3" t="n">
         <v>10</v>
       </c>
-      <c r="P3" t="n">
+      <c r="W3" t="n">
         <v>25</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="X3" t="n">
         <v>5</v>
       </c>
-      <c r="R3" t="n">
+      <c r="Y3" t="n">
         <v>2</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>40</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>24</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -2205,58 +2315,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MODEL</t>
+          <t>BUS_IDX</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>STARTUP</t>
+          <t>PMAX</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>SHUTDOWN</t>
+          <t>CURTAIL_COST</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>ORDER</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>SECOND</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>FIRST</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>ZERO</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>STORAGE</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>RD_UP</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>RD_DOWN</t>
+          <t>STATUS</t>
         </is>
       </c>
     </row>
@@ -2265,63 +2345,27 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>60</v>
+        <v>140</v>
       </c>
       <c r="C2" t="n">
-        <v>10</v>
+        <v>64.05180205514833</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H2" t="n">
-        <v>20</v>
-      </c>
-      <c r="I2" t="n">
-        <v>26</v>
-      </c>
-      <c r="J2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B3" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>56.41707156887287</v>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>6</v>
-      </c>
-      <c r="G3" t="n">
-        <v>40</v>
-      </c>
-      <c r="H3" t="n">
-        <v>40</v>
-      </c>
-      <c r="I3" t="n">
-        <v>24</v>
-      </c>
-      <c r="J3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2335,7 +2379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2362,29 +2406,15 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="C2" t="n">
-        <v>64.05180205514833</v>
+        <v>50.11288767064249</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>8</v>
-      </c>
-      <c r="B3" t="n">
-        <v>150</v>
-      </c>
-      <c r="C3" t="n">
-        <v>56.41707156887287</v>
-      </c>
-      <c r="D3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2399,7 +2429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2415,7 +2445,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>CURTAIL_COST</t>
+          <t>SHED_COST</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -2426,15 +2456,155 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B2" t="n">
+        <v>14.2019305019305</v>
+      </c>
+      <c r="C2" t="n">
+        <v>104.8943261345365</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B3" t="n">
+        <v>68.68146718146718</v>
+      </c>
+      <c r="C3" t="n">
+        <v>118.4132261153868</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="n">
+        <v>50.52162162162162</v>
+      </c>
+      <c r="C4" t="n">
+        <v>115.441479601647</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B5" t="n">
+        <v>20.95366795366795</v>
+      </c>
+      <c r="C5" t="n">
+        <v>100.9991969651695</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B6" t="n">
+        <v>34.68996138996139</v>
+      </c>
+      <c r="C6" t="n">
+        <v>105.3196002843678</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="n">
+        <v>17.69420849420849</v>
+      </c>
+      <c r="C7" t="n">
+        <v>113.8624312652051</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
         <v>6</v>
       </c>
-      <c r="B2" t="n">
-        <v>120</v>
-      </c>
-      <c r="C2" t="n">
-        <v>50.11288767064249</v>
-      </c>
-      <c r="D2" t="n">
+      <c r="B8" t="n">
+        <v>26.07567567567568</v>
+      </c>
+      <c r="C8" t="n">
+        <v>111.7125581799725</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>13</v>
+      </c>
+      <c r="B9" t="n">
+        <v>31.43050193050193</v>
+      </c>
+      <c r="C9" t="n">
+        <v>83.96351606174403</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" t="n">
+        <v>111.2872586872587</v>
+      </c>
+      <c r="C10" t="n">
+        <v>85.3097348506417</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>11</v>
+      </c>
+      <c r="B11" t="n">
+        <v>8.148648648648649</v>
+      </c>
+      <c r="C11" t="n">
+        <v>92.26434686590778</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B12" t="n">
+        <v>219.3150579150579</v>
+      </c>
+      <c r="C12" t="n">
+        <v>99.05190169354194</v>
+      </c>
+      <c r="D12" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2449,183 +2619,63 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BUS_IDX</t>
+          <t>KEY</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>PMAX</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>SHED_COST</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>STATUS</t>
+          <t>VALUE</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B2" t="n">
-        <v>14.2019305019305</v>
-      </c>
-      <c r="C2" t="n">
-        <v>104.8943261345365</v>
-      </c>
-      <c r="D2" t="n">
-        <v>1</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>schema_version</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>9</v>
-      </c>
-      <c r="B3" t="n">
-        <v>68.68146718146718</v>
-      </c>
-      <c r="C3" t="n">
-        <v>118.4132261153868</v>
-      </c>
-      <c r="D3" t="n">
-        <v>1</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>pypower_case_name</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>case14</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>2</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>baseMVA</t>
+        </is>
       </c>
       <c r="B4" t="n">
-        <v>50.52162162162162</v>
-      </c>
-      <c r="C4" t="n">
-        <v>115.441479601647</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>10</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>random_seed</t>
+        </is>
       </c>
       <c r="B5" t="n">
-        <v>20.95366795366795</v>
-      </c>
-      <c r="C5" t="n">
-        <v>100.9991969651695</v>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>14</v>
-      </c>
-      <c r="B6" t="n">
-        <v>34.68996138996139</v>
-      </c>
-      <c r="C6" t="n">
-        <v>105.3196002843678</v>
-      </c>
-      <c r="D6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" t="n">
-        <v>17.69420849420849</v>
-      </c>
-      <c r="C7" t="n">
-        <v>113.8624312652051</v>
-      </c>
-      <c r="D7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" t="n">
-        <v>26.07567567567568</v>
-      </c>
-      <c r="C8" t="n">
-        <v>111.7125581799725</v>
-      </c>
-      <c r="D8" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>13</v>
-      </c>
-      <c r="B9" t="n">
-        <v>31.43050193050193</v>
-      </c>
-      <c r="C9" t="n">
-        <v>83.96351606174403</v>
-      </c>
-      <c r="D9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" t="n">
-        <v>111.2872586872587</v>
-      </c>
-      <c r="C10" t="n">
-        <v>85.3097348506417</v>
-      </c>
-      <c r="D10" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>11</v>
-      </c>
-      <c r="B11" t="n">
-        <v>8.148648648648649</v>
-      </c>
-      <c r="C11" t="n">
-        <v>92.26434686590778</v>
-      </c>
-      <c r="D11" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>3</v>
-      </c>
-      <c r="B12" t="n">
-        <v>219.3150579150579</v>
-      </c>
-      <c r="C12" t="n">
-        <v>99.05190169354194</v>
-      </c>
-      <c r="D12" t="n">
-        <v>1</v>
+        <v>404</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: update bus configuration and enhance data assignment process
</commit_message>
<xml_diff>
--- a/examples/14bus_uc/14bus_config.xlsx
+++ b/examples/14bus_uc/14bus_config.xlsx
@@ -23,16 +23,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -43,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -51,21 +48,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,67 +423,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>BUS_IDX</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>BUS_TYPE</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>PD</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>QD</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>GS</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>BS</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>BUS_AREA</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>VM</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>VA</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>BASEKV</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>ZONE</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>VMAX</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>VMIN</t>
         </is>
@@ -1090,142 +1078,142 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>BUS_IDX</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>PG</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>QG</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>QMAX</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>QMIN</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>VG</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>MBASE</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>STATUS</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>PMAX</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>PMIN</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>COST_MODEL</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>COST_STARTUP</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>COST_SHUTDOWN</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>COST_ORDER</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>COST_SECOND</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>COST_FIRST</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>COST_ZERO</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>RAMP_UP</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>RAMP_DOWN</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>RAMP_STARTUP</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>RAMP_SHUTDOWN</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>RAMP_UP_RD</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>RAMP_DOWN_RD</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>MIN_ON_TIME</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>MIN_OFF_TIME</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>COST_STORAGE</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>COST_RD_UP</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>COST_RD_DOWN</t>
         </is>
@@ -1418,67 +1406,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>F_BUS_IDX</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>T_BUS_IDX</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>BR_R</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>BR_X</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>BR_B</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>RATE_A</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>RATE_B</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>RATE_C</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>TAP</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>SHIFT</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>STATUS</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>ANGMIN</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>ANGMAX</t>
         </is>
@@ -1501,7 +1489,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>130.3097734383326</v>
+        <v>129.4229440691038</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -1542,7 +1530,7 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>64.14423337174171</v>
+        <v>64.61773381230594</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -1583,7 +1571,7 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>130.2602347430043</v>
+        <v>124.5042533106046</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -1624,7 +1612,7 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>61.16687638555656</v>
+        <v>63.30031400641271</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -1665,7 +1653,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>48.13292922887795</v>
+        <v>48.85418025546216</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -1706,7 +1694,7 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>103.5798292671171</v>
+        <v>96.86761523452502</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -1747,7 +1735,7 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>90.06181033993072</v>
+        <v>93.3379405436764</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -1788,7 +1776,7 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>66.78108966701933</v>
+        <v>57.69904988413388</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -1829,7 +1817,7 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>24.50361692467925</v>
+        <v>30.12454988077816</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -1870,7 +1858,7 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>62.53536899236958</v>
+        <v>64.54614650388923</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -1911,7 +1899,7 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>40.4238514678819</v>
+        <v>41.23767059326343</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -1952,7 +1940,7 @@
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>17.8580050094832</v>
+        <v>18.27965637516219</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -1993,7 +1981,7 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>42.37584802178161</v>
+        <v>43.97525691030005</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
@@ -2075,7 +2063,7 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>118.3264311902259</v>
+        <v>118.8337718520753</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -2116,7 +2104,7 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>32.95419000549958</v>
+        <v>31.78374385844369</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -2157,7 +2145,7 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>33.91572504128086</v>
+        <v>34.02627400550421</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -2198,7 +2186,7 @@
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>36.44927022236042</v>
+        <v>36.2900012255455</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -2280,7 +2268,7 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>33.01363503268947</v>
+        <v>33.61053164114362</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -2319,22 +2307,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>BUS_IDX</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>PMAX</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>CURTAIL_COST</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>STATUS</t>
         </is>
@@ -2383,22 +2371,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>BUS_IDX</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>PMAX</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>CURTAIL_COST</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>STATUS</t>
         </is>
@@ -2433,22 +2421,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>BUS_IDX</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>PMAX</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>SHED_COST</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>STATUS</t>
         </is>
@@ -2623,12 +2611,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>KEY</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>VALUE</t>
         </is>

</xml_diff>